<commit_message>
docs(entrega-2): acorta la selección de regresión de V1 a 58 casos
Los casos de prioridad Baja de los módulos que V2 toca se excluyen salvo que
los incluya otra regla (Alta, confirmar un defecto o haber fallado en V1).
Se actualizan el criterio del ADR-027, 03 (md y xlsx) y el README.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/03-seleccion-regresion.xlsx
+++ b/entrega-2/03-seleccion-regresion.xlsx
@@ -1889,19 +1889,15 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>Incluido</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr"/>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>módulo que V2 toca: Registro (V2 suma gasto compartido, aviso de guardado y confirmación de borrado)</t>
+          <t>prioridad Baja en el módulo Registro, que V2 toca: ninguna otra regla la incluye (no es Alta, no confirma un defecto y no falló en V1); conserva el resultado de la ejecución de V1</t>
         </is>
       </c>
     </row>
@@ -2030,19 +2026,15 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>Incluido</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr"/>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>módulo que V2 toca: Registro (V2 suma gasto compartido, aviso de guardado y confirmación de borrado)</t>
+          <t>prioridad Baja en el módulo Registro, que V2 toca: ninguna otra regla la incluye (no es Alta, no confirma un defecto y no falló en V1); conserva el resultado de la ejecución de V1</t>
         </is>
       </c>
     </row>
@@ -2077,19 +2069,15 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
-        <is>
-          <t>Incluido</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>módulo que V2 toca: Registro (V2 suma gasto compartido, aviso de guardado y confirmación de borrado)</t>
+          <t>prioridad Baja en el módulo Registro, que V2 toca: ninguna otra regla la incluye (no es Alta, no confirma un defecto y no falló en V1); conserva el resultado de la ejecución de V1</t>
         </is>
       </c>
     </row>
@@ -2876,19 +2864,15 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G53" s="4" t="inlineStr">
-        <is>
-          <t>Incluido</t>
-        </is>
-      </c>
-      <c r="H53" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr"/>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>módulo que V2 toca: Cuotas (V2 suma la compra en cuotas empezada y la confirmación destructiva)</t>
+          <t>prioridad Baja en el módulo Cuotas, que V2 toca: ninguna otra regla la incluye (no es Alta, no confirma un defecto y no falló en V1); conserva el resultado de la ejecución de V1</t>
         </is>
       </c>
     </row>
@@ -3393,19 +3377,15 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G64" s="4" t="inlineStr">
-        <is>
-          <t>Incluido</t>
-        </is>
-      </c>
-      <c r="H64" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr"/>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>módulo que V2 toca: Monedas (las suscripciones y las deudas en USD usan el tipo de cambio)</t>
+          <t>prioridad Baja en el módulo Monedas, que V2 toca: ninguna otra regla la incluye (no es Alta, no confirma un defecto y no falló en V1); conserva el resultado de la ejecución de V1</t>
         </is>
       </c>
     </row>
@@ -3769,19 +3749,15 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G72" s="4" t="inlineStr">
-        <is>
-          <t>Incluido</t>
-        </is>
-      </c>
-      <c r="H72" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr"/>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>módulo que V2 toca: Resumen (V2 suma el neto de reembolsos, la torta y el detalle de categoría)</t>
+          <t>prioridad Baja en el módulo Resumen, que V2 toca: ninguna otra regla la incluye (no es Alta, no confirma un defecto y no falló en V1); conserva el resultado de la ejecución de V1</t>
         </is>
       </c>
     </row>
@@ -3863,19 +3839,15 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G74" s="4" t="inlineStr">
-        <is>
-          <t>Incluido</t>
-        </is>
-      </c>
-      <c r="H74" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr"/>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>módulo que V2 toca: Resumen (V2 suma el neto de reembolsos, la torta y el detalle de categoría)</t>
+          <t>prioridad Baja en el módulo Resumen, que V2 toca: ninguna otra regla la incluye (no es Alta, no confirma un defecto y no falló en V1); conserva el resultado de la ejecución de V1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(entrega-2): confirmación de los 22 defectos de V1 sobre V2
Se repiten los pasos de cada defecto de V1 «corregido, falta confirmación»
(DEF-005 a DEF-028, salvo los ya cerrados) con Playwright contra la
aplicación y Supabase locales: 21 quedan confirmados corregidos y 1 no es
concluyente (DEF-023, intermitente: 16 altas sin falla no lo descartan).

El resultado y la evidencia de cada uno están en 03-seleccion-regresion
(sección 5, md y xlsx). Se actualizan el criterio de salida 5 y los desvíos de
06 y el README. Falta ejecutar la regresión de los casos de V1 seleccionados.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/03-seleccion-regresion.xlsx
+++ b/entrega-2/03-seleccion-regresion.xlsx
@@ -34,7 +34,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -54,6 +54,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -96,6 +101,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3956,7 +3964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3965,6 +3973,7 @@
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="90" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4002,7 +4011,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Resultado de la confirmación</t>
+          <t>Resultado de la confirmación (2026-10-28)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Evidencia</t>
         </is>
       </c>
     </row>
@@ -4032,9 +4046,14 @@
           <t>CP-ACC-004</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Contra Supabase Auth local: crear una cuenta con «abc1234» y con «abcdefgh» responde HTTP 422 (weak_password) en las dos.</t>
         </is>
       </c>
     </row>
@@ -4064,9 +4083,14 @@
           <t>CP-CFG-004</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>El movimiento muestra: «Entretenimiento archivada Efectivo -$8.000,00»</t>
         </is>
       </c>
     </row>
@@ -4096,9 +4120,14 @@
           <t>CP-REG-012</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Activos tras eliminar: 0. En «Eliminados» se ve «Martes 20 de octubre Indumentaria eliminada Efectivo -$50.000,00» con botón «Restaurar»</t>
         </is>
       </c>
     </row>
@@ -4128,9 +4157,14 @@
           <t>CP-ACC-002</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Sin sesión redirige a /login?next=%2Fdashboard%3Fperiod%3D2026-06; después de entrar termina en /dashboard?period=2026-06</t>
         </is>
       </c>
     </row>
@@ -4160,9 +4194,14 @@
           <t>CP-CUO-003</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Con una compra en 3 cuotas, cambiar la cuenta «Tarjeta de crédito» a efectivo por API responde HTTP 400 (I6: la cuenta tiene compras en cuotas, no puede dejar de ser tarjeta de crédito) y la cuenta sigue siendo tarjeta de crédito.</t>
         </is>
       </c>
     </row>
@@ -4192,9 +4231,14 @@
           <t>Repetir los pasos del reporte (sin caso propio)</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Tras archivar las 8 y abrir Registrar (dos veces): 0 categorías activas, 8 en total</t>
         </is>
       </c>
     </row>
@@ -4224,9 +4268,14 @@
           <t>CP-CFG-006</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>La lista de cuentas tiene 5 botones «Editar» y 5 «Archivar» (una por cuenta)</t>
         </is>
       </c>
     </row>
@@ -4256,9 +4305,14 @@
           <t>CP-REG-010</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Con 1.000.000.000.000 «Siguiente» queda deshabilitado y aparece el aviso «El monto máximo es $999.999.999.999,99».</t>
         </is>
       </c>
     </row>
@@ -4288,9 +4342,14 @@
           <t>CP-REG-011</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Con US$0,01 a tipo de cambio 0,01 «Siguiente» queda deshabilitado y se ve «En pesos daría menos de $0,01.».</t>
         </is>
       </c>
     </row>
@@ -4320,9 +4379,14 @@
           <t>CP-DAS-003</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Con ?period=0000-01 no hay error; la dirección pasa a /dashboard?period=2026-10 y el mes es Octubre 2026</t>
         </is>
       </c>
     </row>
@@ -4352,9 +4416,14 @@
           <t>Repetir los pasos del reporte (sin caso propio)</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>10 botones de color con data-testid; 8 botones «Editar» con identificador distinto en cada fila</t>
         </is>
       </c>
     </row>
@@ -4384,9 +4453,14 @@
           <t>Repetir los pasos del reporte (sin caso propio)</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Gasto de $1.000 con deuda de $400: HTTP 200 (se crea). Con deuda de $1.500: HTTP 400 I7: la deuda no puede superar el monto del gasto</t>
         </is>
       </c>
     </row>
@@ -4416,9 +4490,14 @@
           <t>CP-CFG-010</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Con tipo de cambio 1250,55555 «Siguiente» queda deshabilitado y se ve «Usá hasta 4 decimales».</t>
         </is>
       </c>
     </row>
@@ -4448,9 +4527,14 @@
           <t>CP-CFG-003</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Crear «salud» con «Salud» activa: «Ya existe una categoría activa con ese nombre»; en la lista queda una sola</t>
         </is>
       </c>
     </row>
@@ -4480,9 +4564,14 @@
           <t>CP-MON-003</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>El tipo de cambio sugerido se muestra como «1.250,00»</t>
         </is>
       </c>
     </row>
@@ -4512,9 +4601,14 @@
           <t>Repetir los pasos del reporte (sin caso propio)</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>En Chromium a 390 px de ancho, los montos entran en su casillero ($2.165.003.118,50, $81.818.491.500,00 y $79.653.488.381,50) y no hay scroll horizontal. No se probó en un iPhone con Safari.</t>
         </is>
       </c>
     </row>
@@ -4544,9 +4638,14 @@
           <t>Repetir los pasos del reporte (sin caso propio)</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>No concluyente</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Chromium: 8 de 8 altas llegan a la configuración inicial; WebKit: 8 de 8 altas llegan a la configuración inicial. El defecto era intermitente (2 de 12 en producción con WebKit, 1 de ~80 en local): 16 altas sin fallas no alcanzan para descartarlo</t>
         </is>
       </c>
     </row>
@@ -4576,9 +4675,14 @@
           <t>Repetir los pasos del reporte (sin caso propio)</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>El foco entra al diálogo (true), 6 Tab seguidos no salen de él (true), Escape lo cierra (true) y el foco queda en «settings-accounts-delete»</t>
         </is>
       </c>
     </row>
@@ -4608,9 +4712,14 @@
           <t>CP-CFG-003</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>El aviso «Esta cuenta tiene compras en cuotas: tiene que seguir siendo tarjeta de crédito» aparece junto a la fila que se edita (a 100 px; pantalla de 812 px)</t>
         </is>
       </c>
     </row>
@@ -4640,9 +4749,14 @@
           <t>Repetir los pasos del reporte (sin caso propio)</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Con las 8 categorías archivadas, Registrar dice «No tenés categorías activas. Creá una o reactivá una archivada en Ajustes.» con enlace a Ajustes, y Ajustes muestra «Archivadas» con un botón para reactivar cada una (8). No se revisó el paso «Tus categorías» de la configuración inicial.</t>
         </is>
       </c>
     </row>
@@ -4672,9 +4786,14 @@
           <t>Repetir los pasos del reporte (sin caso propio)</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Con un 429 simulado la pantalla dice: «Demasiados intentos. Esperá unos minutos antes de volver a intentar»</t>
         </is>
       </c>
     </row>
@@ -4704,9 +4823,14 @@
           <t>Repetir los pasos del reporte (sin caso propio)</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Con la siembra demorada (cuentas 4 s, categorías 1,5 s) Registrar muestra 5 cuentas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: cierra los 22 defectos de V1 confirmados sobre V2, incluido DEF-023
Los estados de DEF-005 a DEF-028 (los que estaban «corregido, falta
confirmación») pasan a «Cerrado» en entrega-1/04-reportes-de-defectos.md.
DEF-023 se cierra por decisión del equipo aunque la confirmación fue no
concluyente (era intermitente; se reabre si reaparece), y así queda dicho en
03, 06 y el README de la entrega 2.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/03-seleccion-regresion.xlsx
+++ b/entrega-2/03-seleccion-regresion.xlsx
@@ -4640,12 +4640,12 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>No concluyente</t>
+          <t>No concluyente (cerrado por decisión del equipo)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Chromium: 8 de 8 altas llegan a la configuración inicial; WebKit: 8 de 8 altas llegan a la configuración inicial. El defecto era intermitente (2 de 12 en producción con WebKit, 1 de ~80 en local): 16 altas sin fallas no alcanzan para descartarlo</t>
+          <t>Chromium: 8 de 8 altas llegan a la configuración inicial; WebKit: 8 de 8 altas llegan a la configuración inicial. El defecto era intermitente (2 de 12 en producción con WebKit, 1 de ~80 en local): 16 altas sin fallas no alcanzan para descartarlo El equipo decidió cerrarlo igual; se reabre si reaparece.</t>
         </is>
       </c>
     </row>

</xml_diff>